<commit_message>
🔒 [FULL] Daily chip data 2026-10-02 23:03
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-10.xlsx
+++ b/data/reports/chip_radar_2026-10.xlsx
@@ -7359,7 +7359,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="B3" s="101" t="inlineStr">
         <is>
-          <t>大牌分析師 近 114/114 交易日出手 5460 次 (695 檔), 風格分布: 隔日沖近似 36% / 當沖 12% / 留倉 51%, 漲停命中 2% (其中 🔒鎖漲停 3%), 前 5 大集中 18%, 長線部位 80% (116 檔), ⚠️ 處置股部位 4% (24 檔), 📦 連續囤貨 62 檔 (最長 17 天 00918, 皆已停止)。 主軸: 📈 長線持有/分散布局/高頻交易/持續進場。</t>
+          <t>大牌分析師 近 114/114 交易日出手 5460 次 (695 檔), 風格分布: 隔日沖近似 36% / 當沖 12% / 留倉 51%, 漲停命中 2% (其中 🔒鎖漲停 3%), 前 5 大集中 18%, 長線部位 80% (116 檔), ⚠️ 處置股部位 3% (20 檔), 📦 連續囤貨 62 檔 (最長 17 天 00918, 皆已停止)。 主軸: 📈 長線持有/分散布局/高頻交易/持續進場。</t>
         </is>
       </c>
     </row>
@@ -27907,7 +27907,7 @@
     <row r="539" ht="16.5" customHeight="1">
       <c r="A539" s="223" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-10-02 21:41 TW | 17/17 success | 來源: 富邦17/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-10-02 23:03 TW | 17/17 success | 來源: 富邦17/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-10-03 03:49
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-10.xlsx
+++ b/data/reports/chip_radar_2026-10.xlsx
@@ -1758,7 +1758,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>💡 🎯 quad 進場 (實測 38.8%, 對照 44.0% 未達顯著): 2330 / 6274 / 2308 +3  |  📌 一般共識: 2454  |  避開 — 除權息 1 檔: 6834 | 明日恐處置 3 檔: 3625/4304/4971  |  訊號: 強偏多 (Q5 81.7%, hot=12)</t>
+          <t>💡 🎯 quad 進場 (實測 38.8%, 對照 44.0% 未達顯著): 2330 / 6274 / 2308 +3  |  📌 一般共識: 2454  |  避開 — 明日恐處置 3 檔: 3625/4304/4971  |  訊號: 強偏多 (Q5 81.7%, hot=12)</t>
         </is>
       </c>
     </row>
@@ -3813,7 +3813,7 @@
     <row r="80" ht="22" customHeight="1">
       <c r="B80" s="58" t="inlineStr">
         <is>
-          <t>▍ G. 注意股 (資料日 20261002)</t>
+          <t>▍ G. 注意股 (資料日 20261003)</t>
         </is>
       </c>
     </row>
@@ -4211,7 +4211,7 @@
     <row r="102" ht="22" customHeight="1">
       <c r="B102" s="65" t="inlineStr">
         <is>
-          <t>▍ I. 未來 30 天除權息 (有效 57 檔, 已剔除過期)</t>
+          <t>▍ I. 未來 30 天除權息 (有效 58 檔, 已剔除過期)</t>
         </is>
       </c>
     </row>
@@ -4245,26 +4245,26 @@
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
-          <t>20261002</t>
+          <t>20261005</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>6834</t>
+          <t>00406A</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>天二科技</t>
+          <t>主動中信台灣收益</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>權</t>
+          <t>息</t>
         </is>
       </c>
       <c r="F104" t="n">
-        <v>0</v>
+        <v>0.138</v>
       </c>
     </row>
     <row r="105">
@@ -4275,12 +4275,12 @@
       </c>
       <c r="C105" s="40" t="inlineStr">
         <is>
-          <t>00406A</t>
+          <t>00939</t>
         </is>
       </c>
       <c r="D105" s="40" t="inlineStr">
         <is>
-          <t>主動中信台灣收益</t>
+          <t>統一台灣高息動能</t>
         </is>
       </c>
       <c r="E105" s="40" t="inlineStr">
@@ -4289,7 +4289,7 @@
         </is>
       </c>
       <c r="F105" s="40" t="n">
-        <v>0.138</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="106">
@@ -4300,12 +4300,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>00939</t>
+          <t>00984D</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>統一台灣高息動能</t>
+          <t>主動聯博全球非投</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -4314,32 +4314,32 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>0.125</v>
+        <v>0.08500000000000001</v>
       </c>
     </row>
     <row r="107">
       <c r="B107" s="40" t="inlineStr">
         <is>
-          <t>20261005</t>
+          <t>20261006</t>
         </is>
       </c>
       <c r="C107" s="40" t="inlineStr">
         <is>
-          <t>00984D</t>
+          <t>2614</t>
         </is>
       </c>
       <c r="D107" s="40" t="inlineStr">
         <is>
-          <t>主動聯博全球非投</t>
+          <t>東森</t>
         </is>
       </c>
       <c r="E107" s="40" t="inlineStr">
         <is>
-          <t>息</t>
+          <t>權息</t>
         </is>
       </c>
       <c r="F107" s="40" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="108">
@@ -4350,47 +4350,45 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2614</t>
+          <t>8021</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>東森</t>
+          <t>尖點</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>權息</t>
+          <t>權</t>
         </is>
       </c>
       <c r="F108" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109">
       <c r="B109" s="40" t="inlineStr">
         <is>
-          <t>20261006</t>
+          <t>20261007</t>
         </is>
       </c>
       <c r="C109" s="40" t="inlineStr">
         <is>
-          <t>8021</t>
+          <t>00940</t>
         </is>
       </c>
       <c r="D109" s="40" t="inlineStr">
         <is>
-          <t>尖點</t>
+          <t>元大台灣價值高息</t>
         </is>
       </c>
       <c r="E109" s="40" t="inlineStr">
         <is>
-          <t>權</t>
-        </is>
-      </c>
-      <c r="F109" s="40" t="n">
-        <v>0</v>
-      </c>
+          <t>息</t>
+        </is>
+      </c>
+      <c r="F109" s="40" t="n"/>
     </row>
     <row r="110">
       <c r="B110" t="inlineStr">
@@ -4400,12 +4398,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>00940</t>
+          <t>00946</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>元大台灣價值高息</t>
+          <t>群益科技高息成長</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -4422,12 +4420,12 @@
       </c>
       <c r="C111" s="40" t="inlineStr">
         <is>
-          <t>00946</t>
+          <t>00953B</t>
         </is>
       </c>
       <c r="D111" s="40" t="inlineStr">
         <is>
-          <t>群益科技高息成長</t>
+          <t>群益優選非投等債</t>
         </is>
       </c>
       <c r="E111" s="40" t="inlineStr">
@@ -4445,12 +4443,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>00953B</t>
+          <t>00985B</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>群益優選非投等債</t>
+          <t>群益ESG投等債0-5</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -4467,20 +4465,22 @@
       </c>
       <c r="C113" s="40" t="inlineStr">
         <is>
-          <t>00985B</t>
+          <t>2890</t>
         </is>
       </c>
       <c r="D113" s="40" t="inlineStr">
         <is>
-          <t>群益ESG投等債0-5</t>
+          <t>永豐金</t>
         </is>
       </c>
       <c r="E113" s="40" t="inlineStr">
         <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F113" s="40" t="n"/>
+          <t>權</t>
+        </is>
+      </c>
+      <c r="F113" s="40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="114">
       <c r="B114" t="inlineStr">
@@ -4490,21 +4490,21 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2890</t>
+          <t>6108</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>永豐金</t>
+          <t>競國</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>權</t>
+          <t>息</t>
         </is>
       </c>
       <c r="F114" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="115">
@@ -4515,12 +4515,12 @@
       </c>
       <c r="C115" s="40" t="inlineStr">
         <is>
-          <t>6108</t>
+          <t>6947</t>
         </is>
       </c>
       <c r="D115" s="40" t="inlineStr">
         <is>
-          <t>競國</t>
+          <t>台鎔科技</t>
         </is>
       </c>
       <c r="E115" s="40" t="inlineStr">
@@ -4529,71 +4529,70 @@
         </is>
       </c>
       <c r="F115" s="40" t="n">
-        <v>1</v>
+        <v>0.533326</v>
       </c>
     </row>
     <row r="116">
       <c r="B116" t="inlineStr">
         <is>
-          <t>20261007</t>
+          <t>20261008</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>6947</t>
+          <t>00400A</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>台鎔科技</t>
+          <t>主動國泰動能高息</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
           <t>息</t>
         </is>
-      </c>
-      <c r="F116" t="n">
-        <v>0.533326</v>
       </c>
     </row>
     <row r="117">
       <c r="B117" s="40" t="inlineStr">
         <is>
-          <t>20261008</t>
+          <t>20261012</t>
         </is>
       </c>
       <c r="C117" s="40" t="inlineStr">
         <is>
-          <t>00400A</t>
+          <t>1449</t>
         </is>
       </c>
       <c r="D117" s="40" t="inlineStr">
         <is>
-          <t>主動國泰動能高息</t>
+          <t>佳和</t>
         </is>
       </c>
       <c r="E117" s="40" t="inlineStr">
         <is>
-          <t>息</t>
-        </is>
-      </c>
-      <c r="F117" s="40" t="n"/>
+          <t>權</t>
+        </is>
+      </c>
+      <c r="F117" s="40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="118">
       <c r="B118" t="inlineStr">
         <is>
-          <t>20261012</t>
+          <t>20261013</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>1449</t>
+          <t>1727</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>佳和</t>
+          <t>中華化</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -4973,9 +4972,9 @@
       </c>
     </row>
     <row r="41">
-      <c r="C41" s="69" t="inlineStr">
-        <is>
-          <t>除權息 1 檔 (6834)</t>
+      <c r="C41" s="71" t="inlineStr">
+        <is>
+          <t>今日無除權息</t>
         </is>
       </c>
     </row>
@@ -27907,7 +27906,7 @@
     <row r="539" ht="16.5" customHeight="1">
       <c r="A539" s="223" t="inlineStr">
         <is>
-          <t>ⓘ top-buyer 資料 fetched @ 2026-10-03 02:50 TW | 17/17 success | 來源: 富邦17/histock0</t>
+          <t>ⓘ top-buyer 資料 fetched @ 2026-10-03 03:49 TW | 17/17 success | 來源: 富邦17/histock0</t>
         </is>
       </c>
     </row>

</xml_diff>